<commit_message>
Rename source sheet to All Data in workbook and narration script
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UzWaHKqwMqxC8VSx43CvCa
</commit_message>
<xml_diff>
--- a/excel-summary-tutorial/Raw_Data_to_Summary.xlsx
+++ b/excel-summary-tutorial/Raw_Data_to_Summary.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -176,7 +176,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OldData" displayName="OldData" ref="A1:F11" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AllData" displayName="AllData" ref="A1:F11" headerRowCount="1">
   <autoFilter ref="A1:F11"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Date"/>
@@ -862,15 +862,15 @@
         </is>
       </c>
       <c r="C3" s="7">
-        <f>SUMIFS('Old Data'!$D:$D,'Old Data'!$B:$B,$A3,'Old Data'!$C:$C,$B3)</f>
+        <f>SUMIFS('All Data'!$D:$D,'All Data'!$B:$B,$A3,'All Data'!$C:$C,$B3)</f>
         <v/>
       </c>
       <c r="D3" s="7">
-        <f>SUMIFS('Old Data'!$E:$E,'Old Data'!$B:$B,$A3,'Old Data'!$C:$C,$B3)</f>
+        <f>SUMIFS('All Data'!$E:$E,'All Data'!$B:$B,$A3,'All Data'!$C:$C,$B3)</f>
         <v/>
       </c>
       <c r="E3" s="7">
-        <f>SUMIFS('Old Data'!$F:$F,'Old Data'!$B:$B,$A3,'Old Data'!$C:$C,$B3)</f>
+        <f>SUMIFS('All Data'!$F:$F,'All Data'!$B:$B,$A3,'All Data'!$C:$C,$B3)</f>
         <v/>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -879,15 +879,15 @@
         </is>
       </c>
       <c r="H3" s="7">
-        <f>SUMIF('Old Data'!$B:$B,$G3,'Old Data'!$D:$D)</f>
+        <f>SUMIF('All Data'!$B:$B,$G3,'All Data'!$D:$D)</f>
         <v/>
       </c>
       <c r="I3" s="7">
-        <f>SUMIF('Old Data'!$B:$B,$G3,'Old Data'!$E:$E)</f>
+        <f>SUMIF('All Data'!$B:$B,$G3,'All Data'!$E:$E)</f>
         <v/>
       </c>
       <c r="J3" s="7">
-        <f>SUMIF('Old Data'!$B:$B,$G3,'Old Data'!$F:$F)</f>
+        <f>SUMIF('All Data'!$B:$B,$G3,'All Data'!$F:$F)</f>
         <v/>
       </c>
     </row>
@@ -903,15 +903,15 @@
         </is>
       </c>
       <c r="C4" s="7">
-        <f>SUMIFS('Old Data'!$D:$D,'Old Data'!$B:$B,$A4,'Old Data'!$C:$C,$B4)</f>
+        <f>SUMIFS('All Data'!$D:$D,'All Data'!$B:$B,$A4,'All Data'!$C:$C,$B4)</f>
         <v/>
       </c>
       <c r="D4" s="7">
-        <f>SUMIFS('Old Data'!$E:$E,'Old Data'!$B:$B,$A4,'Old Data'!$C:$C,$B4)</f>
+        <f>SUMIFS('All Data'!$E:$E,'All Data'!$B:$B,$A4,'All Data'!$C:$C,$B4)</f>
         <v/>
       </c>
       <c r="E4" s="7">
-        <f>SUMIFS('Old Data'!$F:$F,'Old Data'!$B:$B,$A4,'Old Data'!$C:$C,$B4)</f>
+        <f>SUMIFS('All Data'!$F:$F,'All Data'!$B:$B,$A4,'All Data'!$C:$C,$B4)</f>
         <v/>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -920,15 +920,15 @@
         </is>
       </c>
       <c r="H4" s="7">
-        <f>SUMIF('Old Data'!$B:$B,$G4,'Old Data'!$D:$D)</f>
+        <f>SUMIF('All Data'!$B:$B,$G4,'All Data'!$D:$D)</f>
         <v/>
       </c>
       <c r="I4" s="7">
-        <f>SUMIF('Old Data'!$B:$B,$G4,'Old Data'!$E:$E)</f>
+        <f>SUMIF('All Data'!$B:$B,$G4,'All Data'!$E:$E)</f>
         <v/>
       </c>
       <c r="J4" s="7">
-        <f>SUMIF('Old Data'!$B:$B,$G4,'Old Data'!$F:$F)</f>
+        <f>SUMIF('All Data'!$B:$B,$G4,'All Data'!$F:$F)</f>
         <v/>
       </c>
     </row>
@@ -944,15 +944,15 @@
         </is>
       </c>
       <c r="C5" s="7">
-        <f>SUMIFS('Old Data'!$D:$D,'Old Data'!$B:$B,$A5,'Old Data'!$C:$C,$B5)</f>
+        <f>SUMIFS('All Data'!$D:$D,'All Data'!$B:$B,$A5,'All Data'!$C:$C,$B5)</f>
         <v/>
       </c>
       <c r="D5" s="7">
-        <f>SUMIFS('Old Data'!$E:$E,'Old Data'!$B:$B,$A5,'Old Data'!$C:$C,$B5)</f>
+        <f>SUMIFS('All Data'!$E:$E,'All Data'!$B:$B,$A5,'All Data'!$C:$C,$B5)</f>
         <v/>
       </c>
       <c r="E5" s="7">
-        <f>SUMIFS('Old Data'!$F:$F,'Old Data'!$B:$B,$A5,'Old Data'!$C:$C,$B5)</f>
+        <f>SUMIFS('All Data'!$F:$F,'All Data'!$B:$B,$A5,'All Data'!$C:$C,$B5)</f>
         <v/>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -961,15 +961,15 @@
         </is>
       </c>
       <c r="H5" s="7">
-        <f>SUMIF('Old Data'!$B:$B,$G5,'Old Data'!$D:$D)</f>
+        <f>SUMIF('All Data'!$B:$B,$G5,'All Data'!$D:$D)</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>SUMIF('Old Data'!$B:$B,$G5,'Old Data'!$E:$E)</f>
+        <f>SUMIF('All Data'!$B:$B,$G5,'All Data'!$E:$E)</f>
         <v/>
       </c>
       <c r="J5" s="7">
-        <f>SUMIF('Old Data'!$B:$B,$G5,'Old Data'!$F:$F)</f>
+        <f>SUMIF('All Data'!$B:$B,$G5,'All Data'!$F:$F)</f>
         <v/>
       </c>
     </row>
@@ -985,15 +985,15 @@
         </is>
       </c>
       <c r="C6" s="7">
-        <f>SUMIFS('Old Data'!$D:$D,'Old Data'!$B:$B,$A6,'Old Data'!$C:$C,$B6)</f>
+        <f>SUMIFS('All Data'!$D:$D,'All Data'!$B:$B,$A6,'All Data'!$C:$C,$B6)</f>
         <v/>
       </c>
       <c r="D6" s="7">
-        <f>SUMIFS('Old Data'!$E:$E,'Old Data'!$B:$B,$A6,'Old Data'!$C:$C,$B6)</f>
+        <f>SUMIFS('All Data'!$E:$E,'All Data'!$B:$B,$A6,'All Data'!$C:$C,$B6)</f>
         <v/>
       </c>
       <c r="E6" s="7">
-        <f>SUMIFS('Old Data'!$F:$F,'Old Data'!$B:$B,$A6,'Old Data'!$C:$C,$B6)</f>
+        <f>SUMIFS('All Data'!$F:$F,'All Data'!$B:$B,$A6,'All Data'!$C:$C,$B6)</f>
         <v/>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -1026,15 +1026,15 @@
         </is>
       </c>
       <c r="C7" s="7">
-        <f>SUMIFS('Old Data'!$D:$D,'Old Data'!$B:$B,$A7,'Old Data'!$C:$C,$B7)</f>
+        <f>SUMIFS('All Data'!$D:$D,'All Data'!$B:$B,$A7,'All Data'!$C:$C,$B7)</f>
         <v/>
       </c>
       <c r="D7" s="7">
-        <f>SUMIFS('Old Data'!$E:$E,'Old Data'!$B:$B,$A7,'Old Data'!$C:$C,$B7)</f>
+        <f>SUMIFS('All Data'!$E:$E,'All Data'!$B:$B,$A7,'All Data'!$C:$C,$B7)</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>SUMIFS('Old Data'!$F:$F,'Old Data'!$B:$B,$A7,'Old Data'!$C:$C,$B7)</f>
+        <f>SUMIFS('All Data'!$F:$F,'All Data'!$B:$B,$A7,'All Data'!$C:$C,$B7)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch sample stock items to electronics (Laptop, Mobile, Tablet)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UzWaHKqwMqxC8VSx43CvCa
</commit_message>
<xml_diff>
--- a/excel-summary-tutorial/Raw_Data_to_Summary.xlsx
+++ b/excel-summary-tutorial/Raw_Data_to_Summary.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tea Bags</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -557,7 +557,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Green Tea</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -581,7 +581,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tea Bags</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -605,7 +605,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Coffee</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -629,7 +629,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Green Tea</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -653,7 +653,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Coffee</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -677,7 +677,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tea Bags</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -701,7 +701,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Green Tea</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -725,7 +725,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tea Bags</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -749,7 +749,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Coffee</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Tea Bags</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C3" s="7">
@@ -899,7 +899,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Coffee</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C4" s="7">
@@ -940,7 +940,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Green Tea</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="C5" s="7">
@@ -981,7 +981,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Coffee</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="C6" s="7">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Tea Bags</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C7" s="7">

</xml_diff>